<commit_message>
bs_1377_9 (1990, withdrawn) and bs_1377_9_2025 added to the specification registry; roles gains approver
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/roles.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/roles.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9900" yWindow="3640" windowWidth="34440" windowHeight="20320" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lists" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="19.1640625" customWidth="1" style="13" min="1" max="1"/>
@@ -1442,6 +1442,33 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>approver</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Approver</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Person or organization that approved the associated data, document or work - for example a calibration certificate, a test report or an inspection.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -1457,7 +1484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="7.1640625" customWidth="1" style="15" min="1" max="1"/>
@@ -1910,6 +1937,18 @@
         </is>
       </c>
       <c r="C27" t="inlineStr">
+        <is>
+          <t>//diggs:rolePerformed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>approver</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>//diggs:rolePerformed</t>
         </is>

</xml_diff>

<commit_message>
PIT3: roles - data_interpreter (the person or organization that evaluated a recorded signal or measurement record)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/roles.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/roles.xlsx
@@ -782,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="19.1640625" customWidth="1" style="13" min="1" max="1"/>
@@ -1469,6 +1469,33 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>data_interpreter</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Data Interpreter</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Person or organization that evaluated a recorded signal or measurement record to state a result - for example the interpretation of a low strain integrity test record.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
@@ -1484,7 +1511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16"/>
   <cols>
     <col width="7.1640625" customWidth="1" style="15" min="1" max="1"/>
@@ -1949,6 +1976,18 @@
         </is>
       </c>
       <c r="C28" t="inlineStr">
+        <is>
+          <t>//diggs:rolePerformed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>data_interpreter</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
         <is>
           <t>//diggs:rolePerformed</t>
         </is>

</xml_diff>